<commit_message>
List max update to schedule
</commit_message>
<xml_diff>
--- a/ids540_specific/class_schedule_540_xlsx.xlsx
+++ b/ids540_specific/class_schedule_540_xlsx.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10917"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nce8/github/practicaldatascience_book/ids540_specific/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vesper/Documents/GitHub/practicaldatascience_book/ids540_specific/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{115D048C-C7E9-824D-B828-C341FD5A6742}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7CE5677-63B3-794D-B974-7E376B7C3392}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -371,9 +371,6 @@
     <t>- `Blackjack &lt;../exercises/exercise_blackjack.html&gt;`_</t>
   </si>
   <si>
-    <t>- `List Max &lt;../exercises/exercise_listmax.html&gt;`_</t>
-  </si>
-  <si>
     <t>- `HR Peak &lt;../exercises/exercise_hrpeak.html&gt;`_</t>
   </si>
   <si>
@@ -401,6 +398,10 @@
   </si>
   <si>
     <t>- `Blackjack Extensions &lt;../exercises/exercise_blackjack_extensions.html&gt;`_</t>
+  </si>
+  <si>
+    <t>- `List Max &lt;../exercises/exercise_listmax.html&gt;`_ 
+- `HR Peak &lt;../exercises/exercise_hrpeak.html&gt;`_</t>
   </si>
 </sst>
 </file>
@@ -509,9 +510,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -549,7 +550,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -655,7 +656,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -797,7 +798,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -873,7 +874,7 @@
         <v>11</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>93</v>
@@ -923,7 +924,7 @@
         <v>18</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
@@ -931,7 +932,7 @@
         <v>26</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>20</v>
@@ -945,10 +946,10 @@
         <v>29</v>
       </c>
       <c r="B11" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>102</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="34" customHeight="1" x14ac:dyDescent="0.2">
@@ -962,7 +963,7 @@
         <v>23</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="136" customHeight="1" x14ac:dyDescent="0.2">
@@ -973,7 +974,7 @@
         <v>25</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="57" customHeight="1" x14ac:dyDescent="0.2">
@@ -987,7 +988,7 @@
         <v>28</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="170" customHeight="1" x14ac:dyDescent="0.2">
@@ -1001,7 +1002,7 @@
         <v>31</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">

</xml_diff>